<commit_message>
gradient color_hero-minimal-dark block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 8
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -52,7 +52,7 @@
     <t>content-page</t>
   </si>
   <si>
-    <t>2026-09-24T12:08:41.569Z</t>
+    <t>2026-09-24T14:07:26.592Z</t>
   </si>
   <si>
     <t>Home - Pet Care Network | Destination Pet</t>
@@ -70,7 +70,7 @@
     <t>live-webinar</t>
   </si>
   <si>
-    <t>2026-09-24T12:08:45.757Z</t>
+    <t>2026-09-24T14:07:30.677Z</t>
   </si>
   <si>
     <t>A Series of Webinars | Destination Pet</t>
@@ -88,7 +88,7 @@
     <t>live-webinar/webinar-redirect</t>
   </si>
   <si>
-    <t>2026-09-24T08:14:45.556Z</t>
+    <t>2026-09-24T14:07:09.109Z</t>
   </si>
   <si>
     <t>Webinar Redirect - Destination Pet</t>

</xml_diff>

<commit_message>
2 pages under about-us
Automated migration updates generated by Experience Modernization Agent.

Changed files: 12
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="45">
   <si>
     <t>_reportFile</t>
   </si>
@@ -110,6 +110,42 @@
   </si>
   <si>
     <t>https://www.destinationpet.com/live-webinar/webinars-for-pet/</t>
+  </si>
+  <si>
+    <t>about-us/meet-the-team/business-development-leaders.report.json</t>
+  </si>
+  <si>
+    <t>["hero-minimal-dark","columns-comfortable-light","columns-comfortable-light","columns-comfortable-light","columns-comfortable-light"]</t>
+  </si>
+  <si>
+    <t>about-us/meet-the-team/business-development-leaders</t>
+  </si>
+  <si>
+    <t>2026-09-24T15:11:42.024Z</t>
+  </si>
+  <si>
+    <t>Business Development Leaders | Destination Pet</t>
+  </si>
+  <si>
+    <t>https://destinationpet.com/about-us/meet-the-team/business-development-leaders/</t>
+  </si>
+  <si>
+    <t>about-us/meet-the-team/leadership.report.json</t>
+  </si>
+  <si>
+    <t>["hero-minimal-dark","columns-comfortable-light","columns-comfortable-light","columns-comfortable-light","columns-comfortable-light","columns-comfortable-light","columns-comfortable-light","columns-comfortable-light"]</t>
+  </si>
+  <si>
+    <t>about-us/meet-the-team/leadership</t>
+  </si>
+  <si>
+    <t>2026-09-24T15:14:32.119Z</t>
+  </si>
+  <si>
+    <t>Leadership - Meet the team | Destination Pet</t>
+  </si>
+  <si>
+    <t>https://destinationpet.com/about-us/meet-the-team/leadership/</t>
   </si>
 </sst>
 </file>
@@ -498,15 +534,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="43" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="31" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="43" customWidth="1"/>
+    <col min="7" max="7" width="48" customWidth="1"/>
     <col min="8" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
@@ -638,6 +672,58 @@
       </c>
       <c r="H5" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" t="s">
+        <v>43</v>
+      </c>
+      <c r="H7" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
life-at-dp & about page
Automated migration updates generated by Experience Modernization Agent.

Changed files: 30
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="84">
   <si>
     <t>_reportFile</t>
   </si>
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero-minimal-dark","columns-comfortable-light","cards","columns-minimal-light","quote","quote"]</t>
+    <t>["hero-minimal-dark","columns-comfortable-light","cards","cards","columns-minimal-light","quote","quote"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>content-page</t>
   </si>
   <si>
-    <t>2026-09-24T14:07:26.592Z</t>
+    <t>2026-09-25T08:05:44.881Z</t>
   </si>
   <si>
     <t>Home - Pet Care Network | Destination Pet</t>
@@ -70,7 +70,7 @@
     <t>live-webinar</t>
   </si>
   <si>
-    <t>2026-09-24T14:07:30.677Z</t>
+    <t>2026-09-25T08:02:35.749Z</t>
   </si>
   <si>
     <t>A Series of Webinars | Destination Pet</t>
@@ -88,7 +88,7 @@
     <t>sell-your-business</t>
   </si>
   <si>
-    <t>2026-09-24T16:25:30.043Z</t>
+    <t>2026-09-25T08:05:53.206Z</t>
   </si>
   <si>
     <t>Sell Your Veterinary | Destination Pet</t>
@@ -97,6 +97,24 @@
     <t>https://destinationpet.com/sell-your-business/</t>
   </si>
   <si>
+    <t>about-us/about.report.json</t>
+  </si>
+  <si>
+    <t>["hero-minimal-dark","columns-comfortable-light","columns-comfortable-light","columns-comfortable-light","columns-comfortable-light","columns-comfortable-light"]</t>
+  </si>
+  <si>
+    <t>about-us/about</t>
+  </si>
+  <si>
+    <t>2026-09-25T08:03:29.978Z</t>
+  </si>
+  <si>
+    <t>About Us | Destination Pet, LLC</t>
+  </si>
+  <si>
+    <t>https://destinationpet.com/about-us/about/</t>
+  </si>
+  <si>
     <t>about-us/get-in-touch.report.json</t>
   </si>
   <si>
@@ -106,7 +124,7 @@
     <t>about-us/get-in-touch</t>
   </si>
   <si>
-    <t>2026-09-24T15:46:54.898Z</t>
+    <t>2026-09-25T08:03:25.813Z</t>
   </si>
   <si>
     <t>Contact Us | Destination Pet, LLC</t>
@@ -121,7 +139,7 @@
     <t>join-our-pack/find-a-veterinary-externship</t>
   </si>
   <si>
-    <t>2026-09-24T16:03:21.285Z</t>
+    <t>2026-09-25T08:03:40.378Z</t>
   </si>
   <si>
     <t>Find a Veterinary Externship - Destination Pet</t>
@@ -130,6 +148,24 @@
     <t>https://destinationpet.com/join-our-pack/find-a-veterinary-externship/</t>
   </si>
   <si>
+    <t>join-our-pack/life-at-dp.report.json</t>
+  </si>
+  <si>
+    <t>["hero-minimal-dark","quote","video","accordion","accordion"]</t>
+  </si>
+  <si>
+    <t>join-our-pack/life-at-dp</t>
+  </si>
+  <si>
+    <t>2026-09-25T08:03:45.562Z</t>
+  </si>
+  <si>
+    <t>life at Destination Pet | Destination Pet</t>
+  </si>
+  <si>
+    <t>https://destinationpet.com/join-our-pack/life-at-dp/</t>
+  </si>
+  <si>
     <t>live-webinar/webinar-redirect.report.json</t>
   </si>
   <si>
@@ -139,7 +175,7 @@
     <t>live-webinar/webinar-redirect</t>
   </si>
   <si>
-    <t>2026-09-24T14:07:09.109Z</t>
+    <t>2026-09-25T08:02:41.623Z</t>
   </si>
   <si>
     <t>Webinar Redirect - Destination Pet</t>
@@ -154,7 +190,7 @@
     <t>live-webinar/webinar-registration</t>
   </si>
   <si>
-    <t>2026-09-24T16:03:40.908Z</t>
+    <t>2026-09-25T08:03:03.479Z</t>
   </si>
   <si>
     <t>Webinar Registration - Destination Pet</t>
@@ -169,7 +205,7 @@
     <t>live-webinar/webinar-viewing-previous</t>
   </si>
   <si>
-    <t>2026-09-24T16:03:30.923Z</t>
+    <t>2026-09-25T08:02:54.887Z</t>
   </si>
   <si>
     <t>Webinar Viewing Previous - Destination Pet</t>
@@ -184,7 +220,7 @@
     <t>live-webinar/webinars-for-pet</t>
   </si>
   <si>
-    <t>2026-09-24T08:14:49.609Z</t>
+    <t>2026-09-25T08:02:46.277Z</t>
   </si>
   <si>
     <t>Webinars for Pet - Destination Pet</t>
@@ -202,7 +238,7 @@
     <t>about-us/meet-the-team/business-development-leaders</t>
   </si>
   <si>
-    <t>2026-09-24T15:11:42.024Z</t>
+    <t>2026-09-25T08:03:09.150Z</t>
   </si>
   <si>
     <t>Business Development Leaders | Destination Pet</t>
@@ -220,7 +256,7 @@
     <t>about-us/meet-the-team/leadership</t>
   </si>
   <si>
-    <t>2026-09-24T15:14:32.119Z</t>
+    <t>2026-09-25T08:03:16.790Z</t>
   </si>
   <si>
     <t>Leadership - Meet the team | Destination Pet</t>
@@ -615,7 +651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -760,10 +796,10 @@
         <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
@@ -772,21 +808,21 @@
         <v>12</v>
       </c>
       <c r="F6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
         <v>41</v>
@@ -812,10 +848,10 @@
         <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -824,24 +860,24 @@
         <v>12</v>
       </c>
       <c r="F8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -850,24 +886,24 @@
         <v>12</v>
       </c>
       <c r="F9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H9" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
@@ -876,24 +912,24 @@
         <v>12</v>
       </c>
       <c r="F10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
@@ -902,21 +938,21 @@
         <v>12</v>
       </c>
       <c r="F11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B12" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="C12" t="s">
         <v>68</v>
@@ -935,6 +971,58 @@
       </c>
       <c r="H12" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C13" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" t="s">
+        <v>75</v>
+      </c>
+      <c r="G13" t="s">
+        <v>76</v>
+      </c>
+      <c r="H13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" t="s">
+        <v>79</v>
+      </c>
+      <c r="C14" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" t="s">
+        <v>81</v>
+      </c>
+      <c r="G14" t="s">
+        <v>82</v>
+      </c>
+      <c r="H14" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>